<commit_message>
demo: walkthrough exercises live table-level repair loop, no-stub guard
- _require_real_react() fails loud unless EscalatingSubagent + TableValidator
  are wired (MCG_SUBAGENT=react + claude CLI/key) — never silently uses the stub
- fix scenario surfaces the per-pass repair log (MCG_REPAIR_LOG)
- react_fix_sampling.xlsx resized to 65 rows so the band verifier is size-gated
  off and the new table-level repair loop does the dtype-mismatch fix
- gitignore the runtime repair_log.jsonl

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_data/react_fix_sampling.xlsx
+++ b/demo_data/react_fix_sampling.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -702,10 +702,8 @@
       <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C22" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -717,10 +715,8 @@
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -732,10 +728,8 @@
       <c r="B24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C24" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -747,10 +741,8 @@
       <c r="B25" t="n">
         <v>5</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C25" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -762,10 +754,8 @@
       <c r="B26" t="n">
         <v>1</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C26" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -777,10 +767,8 @@
       <c r="B27" t="n">
         <v>2</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C27" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -792,10 +780,8 @@
       <c r="B28" t="n">
         <v>3</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C28" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="29">
@@ -807,10 +793,8 @@
       <c r="B29" t="n">
         <v>4</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -822,10 +806,8 @@
       <c r="B30" t="n">
         <v>5</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -837,10 +819,8 @@
       <c r="B31" t="n">
         <v>1</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C31" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -852,10 +832,8 @@
       <c r="B32" t="n">
         <v>2</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C32" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -867,10 +845,8 @@
       <c r="B33" t="n">
         <v>3</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C33" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="34">
@@ -882,10 +858,8 @@
       <c r="B34" t="n">
         <v>4</v>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C34" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="35">
@@ -897,10 +871,8 @@
       <c r="B35" t="n">
         <v>5</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C35" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="36">
@@ -912,10 +884,8 @@
       <c r="B36" t="n">
         <v>1</v>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -927,10 +897,8 @@
       <c r="B37" t="n">
         <v>2</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C37" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -942,10 +910,8 @@
       <c r="B38" t="n">
         <v>3</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C38" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -957,7 +923,396 @@
       <c r="B39" t="n">
         <v>4</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T039</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>T040</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>T041</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>T042</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>T043</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T044</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>5</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T045</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T046</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>T047</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>T048</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>T049</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>T050</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>T051</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>T052</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>T053</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>4</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>T054</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>T055</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>T056</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>T057</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>T058</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>T059</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>T060</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>T061</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>T062</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>T063</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>T064</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>T065</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>pending</t>
         </is>

</xml_diff>